<commit_message>
trying to add gmv generator
</commit_message>
<xml_diff>
--- a/HandleList.xlsx
+++ b/HandleList.xlsx
@@ -14,693 +14,300 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
-    <t>mekeupupup</t>
+    <t>nany_b8</t>
   </si>
   <si>
-    <t>hallie_grace8</t>
+    <t>mamadawnny</t>
+  </si>
+  <si>
+    <t>vibe_with_stephanie</t>
+  </si>
+  <si>
+    <t>rachelandsam_fitness</t>
+  </si>
+  <si>
+    <t>alaina.jinaee</t>
   </si>
   <si>
     <t>allure_fashion</t>
   </si>
   <si>
-    <t>nphiynhi</t>
+    <t>thettravelqueen2</t>
   </si>
   <si>
-    <t>michellesays</t>
+    <t>vilmahidalgo10</t>
   </si>
   <si>
-    <t>itzesantana11</t>
+    <t>maceylianna</t>
   </si>
   <si>
-    <t>itsmekelsc</t>
+    <t>jujubeingdelulu</t>
   </si>
   <si>
-    <t>mikaylanogueira</t>
+    <t>leah_txrealtor</t>
   </si>
   <si>
-    <t>smittyyyyyyy1</t>
+    <t>kylieoguma</t>
   </si>
   <si>
-    <t>itsisabelbedoyaa</t>
+    <t>iamsharihelene</t>
   </si>
   <si>
-    <t>rancobeauty</t>
+    <t>rubyfinds_</t>
   </si>
   <si>
-    <t>lifeaskristinab</t>
+    <t>bettygtz24</t>
   </si>
   <si>
-    <t>ayannasabrina</t>
-  </si>
-  <si>
-    <t>siearaashton</t>
-  </si>
-  <si>
-    <t>beautywithaj</t>
-  </si>
-  <si>
-    <t>miarenaa_</t>
-  </si>
-  <si>
-    <t>ashmartodam</t>
-  </si>
-  <si>
-    <t>nasochami</t>
-  </si>
-  <si>
-    <t>wowvall</t>
-  </si>
-  <si>
-    <t>colleen_fusco</t>
-  </si>
-  <si>
-    <t>makeupartistatlaw</t>
-  </si>
-  <si>
-    <t>mikemorea</t>
-  </si>
-  <si>
-    <t>sam_joness_</t>
-  </si>
-  <si>
-    <t>michaelascott20</t>
-  </si>
-  <si>
-    <t>kaitlynclayton13</t>
-  </si>
-  <si>
-    <t>liceisyummy</t>
-  </si>
-  <si>
-    <t>itsmakeupbymelissam</t>
-  </si>
-  <si>
-    <t>kellyrosesarno</t>
-  </si>
-  <si>
-    <t>gabbysimpson22</t>
-  </si>
-  <si>
-    <t>fentybeauty</t>
-  </si>
-  <si>
-    <t>logantheempress</t>
-  </si>
-  <si>
-    <t>the_makeup_mami</t>
-  </si>
-  <si>
-    <t>sobermakeupmama_paige</t>
-  </si>
-  <si>
-    <t>byfabilicious</t>
-  </si>
-  <si>
-    <t>boomkackmua</t>
-  </si>
-  <si>
-    <t>zarahbutler</t>
-  </si>
-  <si>
-    <t>lorixasiaa</t>
-  </si>
-  <si>
-    <t>thecoachsamantha</t>
-  </si>
-  <si>
-    <t>angelamachadobeauty</t>
-  </si>
-  <si>
-    <t>queencosmeticsofficial</t>
-  </si>
-  <si>
-    <t>loveemanda</t>
-  </si>
-  <si>
-    <t>vprincemusic</t>
-  </si>
-  <si>
-    <t>ghostgirlcosplay2</t>
-  </si>
-  <si>
-    <t>lianet1006</t>
-  </si>
-  <si>
-    <t>ericataylor2347</t>
-  </si>
-  <si>
-    <t>madelynguerreroh</t>
-  </si>
-  <si>
-    <t>kseniasenn</t>
-  </si>
-  <si>
-    <t>dibsbeauty</t>
-  </si>
-  <si>
-    <t>yvettejaninee</t>
-  </si>
-  <si>
-    <t>allithatglitters</t>
-  </si>
-  <si>
-    <t>andreasaraii</t>
-  </si>
-  <si>
-    <t>dazeemaee</t>
-  </si>
-  <si>
-    <t>kaganbrooks</t>
-  </si>
-  <si>
-    <t>ingaterner</t>
-  </si>
-  <si>
-    <t>anitamironbeauty</t>
-  </si>
-  <si>
-    <t>tatiencorea</t>
-  </si>
-  <si>
-    <t>loganwalter05</t>
-  </si>
-  <si>
-    <t>tusister_jurissa</t>
-  </si>
-  <si>
-    <t>siana_far</t>
-  </si>
-  <si>
-    <t>andreaguevara2019</t>
-  </si>
-  <si>
-    <t>veralmakeup</t>
-  </si>
-  <si>
-    <t>pierinamontano</t>
-  </si>
-  <si>
-    <t>humblemenails</t>
-  </si>
-  <si>
-    <t>arianemann</t>
-  </si>
-  <si>
-    <t>shellyseashell1.0</t>
-  </si>
-  <si>
-    <t>haleyparkerstyle</t>
-  </si>
-  <si>
-    <t>arevceline</t>
-  </si>
-  <si>
-    <t>thirtywaves</t>
-  </si>
-  <si>
-    <t>carlosantoniocerv</t>
-  </si>
-  <si>
-    <t>boise_brooke</t>
-  </si>
-  <si>
-    <t>vi0letred</t>
-  </si>
-  <si>
-    <t>bhutekobhat3</t>
-  </si>
-  <si>
-    <t>the_pinder_home</t>
-  </si>
-  <si>
-    <t>whatmandi</t>
-  </si>
-  <si>
-    <t>vanillacrush</t>
-  </si>
-  <si>
-    <t>lifesrad</t>
-  </si>
-  <si>
-    <t>taybeckerbeauty</t>
-  </si>
-  <si>
-    <t>kwital</t>
-  </si>
-  <si>
-    <t>itslunakareem</t>
-  </si>
-  <si>
-    <t>elenaduquebeauty</t>
-  </si>
-  <si>
-    <t>lalamilan</t>
-  </si>
-  <si>
-    <t>officialtinysierra</t>
-  </si>
-  <si>
-    <t>get_glam_with_sadaf</t>
-  </si>
-  <si>
-    <t>notswagpop</t>
-  </si>
-  <si>
-    <t>maya.videodiary</t>
-  </si>
-  <si>
-    <t>domenicadaniela10</t>
-  </si>
-  <si>
-    <t>dr.ljmaxfield</t>
-  </si>
-  <si>
-    <t>the_geriatricmillennial</t>
-  </si>
-  <si>
-    <t>goonza_costa</t>
-  </si>
-  <si>
-    <t>benjaminzamoratv</t>
-  </si>
-  <si>
-    <t>munozpmagally</t>
-  </si>
-  <si>
-    <t>chicoruizzz</t>
-  </si>
-  <si>
-    <t>goodasshairday</t>
-  </si>
-  <si>
-    <t>rachelnoelleclark</t>
-  </si>
-  <si>
-    <t>locks.by.libbybrenner</t>
-  </si>
-  <si>
-    <t>itstiffslife</t>
-  </si>
-  <si>
-    <t>bretmanrock</t>
-  </si>
-  <si>
-    <t>jeremystoomuch</t>
-  </si>
-  <si>
-    <t>jessebaizer</t>
-  </si>
-  <si>
-    <t>veritoomom</t>
-  </si>
-  <si>
-    <t>jorgee.brando</t>
-  </si>
-  <si>
-    <t>real.natalia</t>
-  </si>
-  <si>
-    <t>brothernailtech</t>
+    <t>notk3sa</t>
   </si>
   <si>
     <t>mplyly</t>
   </si>
   <si>
-    <t>dimaggioglows</t>
+    <t>transparent.taylor</t>
   </si>
   <si>
-    <t>jenniixmarie</t>
+    <t>dresswithdiane</t>
   </si>
   <si>
-    <t>rxthism</t>
+    <t>soynoheliaenusa</t>
   </si>
   <si>
-    <t>amandasikoralmusic</t>
+    <t>lovergirlnunu1</t>
   </si>
   <si>
-    <t>theskincarebakery</t>
+    <t>karla_navarro1</t>
   </si>
   <si>
-    <t>terreetaughtme</t>
+    <t>heyitsme.lc</t>
   </si>
   <si>
-    <t>terrykaye</t>
+    <t>the_good_stuff_co</t>
   </si>
   <si>
-    <t>shoelover99</t>
+    <t>puffydesh</t>
   </si>
   <si>
-    <t>tabitha_gonzalez</t>
+    <t>brittainyshaw</t>
   </si>
   <si>
-    <t>normaescandontiktok</t>
+    <t>blessingreviewsthings</t>
   </si>
   <si>
-    <t>mavwicksfragrances</t>
+    <t>jessdoumat</t>
   </si>
   <si>
-    <t>21makeupaddictions</t>
+    <t>keidrabelle</t>
   </si>
   <si>
-    <t>rosekemanuel</t>
+    <t>lexitay_</t>
   </si>
   <si>
-    <t>dermdoctor</t>
+    <t>lexiemcdonald_</t>
   </si>
   <si>
-    <t>jenny_claross</t>
+    <t>hannahsahm</t>
   </si>
   <si>
-    <t>yuni.fitbeauty</t>
+    <t>ohsoitsjocelyn</t>
   </si>
   <si>
-    <t>lorenrosko</t>
+    <t>balliecolleenhart</t>
   </si>
   <si>
-    <t>danielleathena</t>
+    <t>karlitavasquez5031</t>
   </si>
   <si>
-    <t>thezoerenee</t>
+    <t>creatorchristie</t>
   </si>
   <si>
-    <t>dunia_santos_urbina</t>
+    <t>sarahwade275</t>
   </si>
   <si>
-    <t>adryhavana</t>
+    <t>lordkierra</t>
   </si>
   <si>
-    <t>alexa_de</t>
+    <t>flormedrano.21</t>
   </si>
   <si>
-    <t>makaylahelms</t>
+    <t>cab9896</t>
   </si>
   <si>
-    <t>carlos_eduardo_espina</t>
+    <t>ellyevercreations</t>
   </si>
   <si>
-    <t>bryttani_mingo</t>
+    <t>kesha.nikshell</t>
   </si>
   <si>
-    <t>thebentist</t>
+    <t>maryvictoriaf</t>
   </si>
   <si>
-    <t>mrs.isabelabarbosa</t>
+    <t>africanherbswoman</t>
   </si>
   <si>
-    <t>amyjackson9213</t>
+    <t>fw.joanaaa9805</t>
   </si>
   <si>
-    <t>lahony69</t>
+    <t>mafiagodmom</t>
   </si>
   <si>
-    <t>sashacoo1</t>
+    <t>coolk1dmae</t>
   </si>
   <si>
-    <t>karissastevens_</t>
+    <t>captainvalgenae</t>
   </si>
   <si>
-    <t>linds.w11</t>
+    <t>loracroftcheck</t>
   </si>
   <si>
-    <t>tonikohl4</t>
+    <t>ciao_jayc</t>
   </si>
   <si>
-    <t>brrrila</t>
+    <t>oraliamartinez99</t>
   </si>
   <si>
-    <t>jahairaallende</t>
+    <t>cierraryyan</t>
   </si>
   <si>
-    <t>j_okayyy</t>
+    <t>tati_rosalie</t>
   </si>
   <si>
-    <t>aliiceberg</t>
+    <t>lamomdeals</t>
   </si>
   <si>
-    <t>roy_mccarty</t>
+    <t>britneylea19</t>
   </si>
   <si>
-    <t>rafaelmelendez580</t>
+    <t>nathaliarivera</t>
   </si>
   <si>
-    <t>losachos</t>
+    <t>anneallenfloyd</t>
   </si>
   <si>
-    <t>oliviabirrueta</t>
+    <t>ekndra</t>
   </si>
   <si>
-    <t>drew.tts</t>
+    <t>chanandlo</t>
   </si>
   <si>
-    <t>100proofflowfitness</t>
+    <t>zashianahoward</t>
   </si>
   <si>
-    <t>ariugcenthusiast</t>
+    <t>morg_lucas</t>
   </si>
   <si>
-    <t>mattkahla</t>
+    <t>annajones1415</t>
   </si>
   <si>
-    <t>julietsfinds</t>
+    <t>katshopsalot</t>
   </si>
   <si>
-    <t>_graciedavis</t>
+    <t>brittneys.favorite.finds</t>
   </si>
   <si>
-    <t>speedqueenmamma</t>
+    <t>hygienequeen_1</t>
   </si>
   <si>
-    <t>thicwhip</t>
+    <t>bonitajoo</t>
   </si>
   <si>
-    <t>lukasgreyy</t>
+    <t>clipsntea</t>
   </si>
   <si>
-    <t>sheri_pie455</t>
+    <t>mommacasss</t>
   </si>
   <si>
-    <t>pnwdad206</t>
+    <t>nardistoryteller</t>
   </si>
   <si>
-    <t>suzieqssss</t>
+    <t>fierceangellb</t>
   </si>
   <si>
-    <t>mariaalicea0314</t>
+    <t>fannyfuen07</t>
   </si>
   <si>
-    <t>mariomagana2</t>
+    <t>alexia.rose19</t>
   </si>
   <si>
-    <t>alacartaconsabor</t>
+    <t>brendaglams</t>
   </si>
   <si>
-    <t>jaime_kiroz</t>
+    <t>brownsugar_088tts</t>
   </si>
   <si>
-    <t>astringofhope</t>
+    <t>emia_stef</t>
   </si>
   <si>
-    <t>itsambaslife</t>
+    <t>kel.1026</t>
   </si>
   <si>
-    <t>xochitlmakesitneat</t>
+    <t>ivylosada</t>
   </si>
   <si>
-    <t>liz_the_clearancequeen</t>
+    <t>andthatsthelipton</t>
   </si>
   <si>
-    <t>_amourjaaay</t>
+    <t>moriahh51</t>
   </si>
   <si>
-    <t>crystalsehy</t>
+    <t>finejawn98</t>
   </si>
   <si>
-    <t>samanfaaa</t>
+    <t>ncolettem</t>
   </si>
   <si>
-    <t>rubyfinds_</t>
+    <t>localmaani</t>
   </si>
   <si>
-    <t>bellarush</t>
+    <t>sofloridagirl</t>
   </si>
   <si>
-    <t>branchswrldshop</t>
+    <t>theelboogy</t>
   </si>
   <si>
-    <t>dj.foof</t>
+    <t>mariellakarin</t>
   </si>
   <si>
-    <t>noemic503</t>
+    <t>paigemarshall_</t>
   </si>
   <si>
-    <t>alexanderjaneboutique</t>
+    <t>aleksamink</t>
   </si>
   <si>
-    <t>_mily_mily</t>
+    <t>cutlikeagem</t>
   </si>
   <si>
-    <t>kaileesoto_</t>
+    <t>margaritadoesitall</t>
   </si>
   <si>
-    <t>sabrina_guzzardo</t>
+    <t>tania_fashion_girl</t>
   </si>
   <si>
-    <t>calicurvesfajas</t>
+    <t>mamasherresse</t>
   </si>
   <si>
-    <t>tavifitboss</t>
+    <t>lalajohnston</t>
   </si>
   <si>
-    <t>holllynoel</t>
+    <t>hthosttkull</t>
   </si>
   <si>
-    <t>makeupbyjh</t>
+    <t>yeraldy.love3</t>
   </si>
   <si>
-    <t>kristinadunn2.0</t>
+    <t>michellesfaves</t>
   </si>
   <si>
-    <t>wesleyrbarker</t>
+    <t>budgetbabecloset</t>
   </si>
   <si>
-    <t>lifeofyess</t>
+    <t>lindsaydbeauty</t>
   </si>
   <si>
-    <t>chryssyvsdream</t>
-  </si>
-  <si>
-    <t>thnxsatan</t>
-  </si>
-  <si>
-    <t>ninadoesthemost</t>
-  </si>
-  <si>
-    <t>braidsarekey</t>
-  </si>
-  <si>
-    <t>kimakapapi</t>
-  </si>
-  <si>
-    <t>kaliroseboutique</t>
-  </si>
-  <si>
-    <t>torijflow</t>
-  </si>
-  <si>
-    <t>foxandluxe</t>
-  </si>
-  <si>
-    <t>katrinadimiele</t>
-  </si>
-  <si>
-    <t>boldandbeautifulfashion</t>
-  </si>
-  <si>
-    <t>alanary20</t>
-  </si>
-  <si>
-    <t>jos__96</t>
-  </si>
-  <si>
-    <t>zjuiice</t>
-  </si>
-  <si>
-    <t>cherryyberry</t>
-  </si>
-  <si>
-    <t>tamiacyenne</t>
-  </si>
-  <si>
-    <t>titleykm</t>
-  </si>
-  <si>
-    <t>allstyleschanceculp</t>
-  </si>
-  <si>
-    <t>doradamorrobel</t>
-  </si>
-  <si>
-    <t>michoacana2001</t>
-  </si>
-  <si>
-    <t>mayialvarez5</t>
-  </si>
-  <si>
-    <t>amaiaburuchaga</t>
-  </si>
-  <si>
-    <t>carmenann40</t>
-  </si>
-  <si>
-    <t>flavi.lovely</t>
-  </si>
-  <si>
-    <t>saffronshops</t>
-  </si>
-  <si>
-    <t>amanda_hadzimichalis</t>
-  </si>
-  <si>
-    <t>chclaterayne</t>
-  </si>
-  <si>
-    <t>meeshjessicaparker</t>
-  </si>
-  <si>
-    <t>bettygtz24</t>
-  </si>
-  <si>
-    <t>mscrystalmarie88</t>
-  </si>
-  <si>
-    <t>mandapaints</t>
-  </si>
-  <si>
-    <t>deisabelmontes</t>
-  </si>
-  <si>
-    <t>bethanywei</t>
-  </si>
-  <si>
-    <t>mrskariclark</t>
-  </si>
-  <si>
-    <t>talexiajohnson</t>
-  </si>
-  <si>
-    <t>heather.eva</t>
-  </si>
-  <si>
-    <t>irisnicole_1</t>
-  </si>
-  <si>
-    <t>deestarks79</t>
-  </si>
-  <si>
-    <t>amberhaines26</t>
-  </si>
-  <si>
-    <t>lish.ann</t>
-  </si>
-  <si>
-    <t>nelita.tiki</t>
-  </si>
-  <si>
-    <t>lizpineda824</t>
-  </si>
-  <si>
-    <t>almaagee_</t>
-  </si>
-  <si>
-    <t>staygoldlex</t>
-  </si>
-  <si>
-    <t>ashleydawnofficial</t>
-  </si>
-  <si>
-    <t>ladywonder.31</t>
+    <t>kely6941</t>
   </si>
 </sst>
 </file>
@@ -709,11 +316,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -723,7 +330,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -744,13 +351,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="13"/>
       <color theme="3"/>
@@ -759,18 +359,18 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -783,7 +383,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -792,34 +400,6 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -835,15 +415,21 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -857,7 +443,37 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -873,23 +489,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -910,31 +510,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -952,7 +558,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -964,19 +570,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -988,55 +618,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1054,13 +642,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1072,13 +666,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1090,7 +690,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1143,6 +743,30 @@
       <diagonal/>
     </border>
     <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -1158,15 +782,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -1178,32 +793,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1231,123 +820,134 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1356,28 +956,28 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1396,7 +996,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1730,1449 +1330,1065 @@
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:1">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:1">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:1">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:1">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:1">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:1">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:1">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:1">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:1">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:1">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:1">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:1">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:1">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:1">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:1">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:1">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:1">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:1">
-      <c r="A38" s="3" t="s">
+      <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:1">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:1">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:1">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:1">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:1">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:1">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:1">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:1">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:1">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:1">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:1">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:1">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:1">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:1">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:1">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:1">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:1">
-      <c r="A58" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1">
-      <c r="A59" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1">
-      <c r="A60" s="3" t="s">
+      <c r="A58" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="61" spans="1:1">
-      <c r="A61" s="3" t="s">
+    <row r="59" spans="1:1">
+      <c r="A59" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
-      <c r="A62" s="3" t="s">
+    <row r="60" spans="1:1">
+      <c r="A60" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
-      <c r="A63" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1">
-      <c r="A64" s="3" t="s">
+    <row r="61" spans="1:1">
+      <c r="A61" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="65" spans="1:1">
-      <c r="A65" s="3" t="s">
+    <row r="62" spans="1:1">
+      <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="66" spans="1:1">
-      <c r="A66" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1">
-      <c r="A67" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1">
-      <c r="A68" s="3" t="s">
+    <row r="63" spans="1:1">
+      <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="69" spans="1:1">
-      <c r="A69" s="3" t="s">
+    <row r="64" spans="1:1">
+      <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="70" spans="1:1">
-      <c r="A70" s="3" t="s">
+    <row r="65" spans="1:1">
+      <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="71" spans="1:1">
-      <c r="A71" s="3" t="s">
+    <row r="66" spans="1:1">
+      <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="72" spans="1:1">
-      <c r="A72" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1">
-      <c r="A73" s="3" t="s">
+    <row r="67" spans="1:1">
+      <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="74" spans="1:1">
-      <c r="A74" s="3" t="s">
+    <row r="68" spans="1:1">
+      <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="75" spans="1:1">
-      <c r="A75" s="3" t="s">
+    <row r="69" spans="1:1">
+      <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="76" spans="1:1">
-      <c r="A76" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1">
-      <c r="A77" s="3" t="s">
+    <row r="70" spans="1:1">
+      <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="78" spans="1:1">
-      <c r="A78" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1">
-      <c r="A79" s="3" t="s">
+    <row r="71" spans="1:1">
+      <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="80" spans="1:1">
-      <c r="A80" s="3" t="s">
+    <row r="72" spans="1:1">
+      <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
-      <c r="A81" s="3" t="s">
+    <row r="73" spans="1:1">
+      <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
-      <c r="A82" s="3" t="s">
+    <row r="74" spans="1:1">
+      <c r="A74" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="83" spans="1:1">
-      <c r="A83" s="3" t="s">
+    <row r="75" spans="1:1">
+      <c r="A75" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="84" spans="1:1">
-      <c r="A84" s="3" t="s">
+    <row r="76" spans="1:1">
+      <c r="A76" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="85" spans="1:1">
-      <c r="A85" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="86" spans="1:1">
-      <c r="A86" s="3" t="s">
+    <row r="77" spans="1:1">
+      <c r="A77" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="87" spans="1:1">
-      <c r="A87" s="3" t="s">
+    <row r="78" spans="1:1">
+      <c r="A78" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="88" spans="1:1">
-      <c r="A88" s="3" t="s">
+    <row r="79" spans="1:1">
+      <c r="A79" s="2" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="89" spans="1:1">
-      <c r="A89" s="3" t="s">
+    <row r="80" spans="1:1">
+      <c r="A80" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="90" spans="1:1">
-      <c r="A90" s="3" t="s">
+    <row r="81" spans="1:1">
+      <c r="A81" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="91" spans="1:1">
-      <c r="A91" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1">
-      <c r="A92" s="3" t="s">
+    <row r="82" spans="1:1">
+      <c r="A82" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="93" spans="1:1">
-      <c r="A93" s="3" t="s">
+    <row r="83" spans="1:1">
+      <c r="A83" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="94" spans="1:1">
-      <c r="A94" s="3" t="s">
+    <row r="84" spans="1:1">
+      <c r="A84" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="95" spans="1:1">
-      <c r="A95" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1">
-      <c r="A96" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1">
-      <c r="A97" s="3" t="s">
+    <row r="85" spans="1:1">
+      <c r="A85" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="98" spans="1:1">
-      <c r="A98" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="99" spans="1:1">
-      <c r="A99" s="3" t="s">
+    <row r="86" spans="1:1">
+      <c r="A86" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="100" spans="1:1">
-      <c r="A100" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1">
-      <c r="A101" s="3" t="s">
+    <row r="87" spans="1:1">
+      <c r="A87" s="2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="102" spans="1:1">
-      <c r="A102" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1">
-      <c r="A103" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1">
-      <c r="A104" s="3" t="s">
+    <row r="88" spans="1:1">
+      <c r="A88" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="105" spans="1:1">
-      <c r="A105" s="3" t="s">
+    <row r="89" spans="1:1">
+      <c r="A89" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="106" spans="1:1">
-      <c r="A106" s="3" t="s">
+    <row r="90" spans="1:1">
+      <c r="A90" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="107" spans="1:1">
-      <c r="A107" s="3" t="s">
+    <row r="91" spans="1:1">
+      <c r="A91" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="108" spans="1:1">
-      <c r="A108" s="3" t="s">
+    <row r="92" spans="1:1">
+      <c r="A92" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="109" spans="1:1">
-      <c r="A109" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1">
-      <c r="A110" s="3" t="s">
+    <row r="93" spans="1:1">
+      <c r="A93" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="111" spans="1:1">
-      <c r="A111" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1">
-      <c r="A112" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1">
-      <c r="A113" s="3" t="s">
+    <row r="94" spans="1:1">
+      <c r="A94" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="114" spans="1:1">
-      <c r="A114" s="3" t="s">
+    <row r="95" spans="1:1">
+      <c r="A95" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="115" spans="1:1">
-      <c r="A115" s="3" t="s">
+    <row r="96" spans="1:1">
+      <c r="A96" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="116" spans="1:1">
-      <c r="A116" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="117" spans="1:1">
-      <c r="A117" s="3" t="s">
+    <row r="97" spans="1:1">
+      <c r="A97" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="118" spans="1:1">
-      <c r="A118" s="3" t="s">
+    <row r="98" spans="1:1">
+      <c r="A98" s="2" t="s">
         <v>97</v>
       </c>
     </row>
+    <row r="99" spans="1:1">
+      <c r="A99" s="3"/>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" s="3"/>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" s="3"/>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" s="3"/>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" s="3"/>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" s="3"/>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" s="3"/>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" s="3"/>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" s="3"/>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" s="3"/>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" s="3"/>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" s="3"/>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" s="3"/>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" s="3"/>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" s="3"/>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" s="3"/>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" s="3"/>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" s="3"/>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" s="3"/>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" s="3"/>
+    </row>
     <row r="119" spans="1:1">
-      <c r="A119" s="3" t="s">
-        <v>98</v>
-      </c>
+      <c r="A119" s="3"/>
     </row>
     <row r="120" spans="1:1">
-      <c r="A120" s="3" t="s">
-        <v>99</v>
-      </c>
+      <c r="A120" s="3"/>
     </row>
     <row r="121" spans="1:1">
-      <c r="A121" s="3" t="s">
-        <v>100</v>
-      </c>
+      <c r="A121" s="3"/>
     </row>
     <row r="122" ht="15" customHeight="1" spans="1:1">
-      <c r="A122" s="3" t="s">
-        <v>101</v>
-      </c>
+      <c r="A122" s="3"/>
     </row>
     <row r="123" spans="1:1">
-      <c r="A123" s="3" t="s">
-        <v>0</v>
-      </c>
+      <c r="A123" s="3"/>
     </row>
     <row r="124" spans="1:1">
-      <c r="A124" s="3" t="s">
-        <v>102</v>
-      </c>
+      <c r="A124" s="3"/>
     </row>
     <row r="125" spans="1:1">
-      <c r="A125" s="3" t="s">
-        <v>103</v>
-      </c>
+      <c r="A125" s="3"/>
     </row>
     <row r="126" spans="1:1">
-      <c r="A126" s="3" t="s">
-        <v>104</v>
-      </c>
+      <c r="A126" s="3"/>
     </row>
     <row r="127" spans="1:1">
-      <c r="A127" s="3" t="s">
-        <v>105</v>
-      </c>
+      <c r="A127" s="3"/>
     </row>
     <row r="128" spans="1:1">
-      <c r="A128" s="3" t="s">
-        <v>106</v>
-      </c>
+      <c r="A128" s="3"/>
     </row>
     <row r="129" spans="1:1">
-      <c r="A129" s="3" t="s">
-        <v>107</v>
-      </c>
+      <c r="A129" s="3"/>
     </row>
     <row r="130" spans="1:1">
-      <c r="A130" s="3" t="s">
-        <v>108</v>
-      </c>
+      <c r="A130" s="3"/>
     </row>
     <row r="131" spans="1:1">
-      <c r="A131" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="A131" s="3"/>
     </row>
     <row r="132" spans="1:1">
-      <c r="A132" s="3" t="s">
-        <v>110</v>
-      </c>
+      <c r="A132" s="3"/>
     </row>
     <row r="133" spans="1:1">
-      <c r="A133" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="A133" s="3"/>
     </row>
     <row r="134" spans="1:1">
-      <c r="A134" s="3" t="s">
-        <v>112</v>
-      </c>
+      <c r="A134" s="3"/>
     </row>
     <row r="135" spans="1:1">
-      <c r="A135" s="3" t="s">
-        <v>113</v>
-      </c>
+      <c r="A135" s="3"/>
     </row>
     <row r="136" spans="1:1">
-      <c r="A136" s="3" t="s">
-        <v>114</v>
-      </c>
+      <c r="A136" s="3"/>
     </row>
     <row r="137" spans="1:1">
-      <c r="A137" s="3" t="s">
-        <v>115</v>
-      </c>
+      <c r="A137" s="3"/>
     </row>
     <row r="138" spans="1:1">
-      <c r="A138" s="3" t="s">
-        <v>116</v>
-      </c>
+      <c r="A138" s="3"/>
     </row>
     <row r="139" spans="1:1">
-      <c r="A139" s="3" t="s">
-        <v>117</v>
-      </c>
+      <c r="A139" s="3"/>
     </row>
     <row r="140" spans="1:1">
-      <c r="A140" s="3" t="s">
-        <v>118</v>
-      </c>
+      <c r="A140" s="3"/>
     </row>
     <row r="141" spans="1:1">
-      <c r="A141" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A141" s="3"/>
     </row>
     <row r="142" spans="1:1">
-      <c r="A142" s="3" t="s">
-        <v>119</v>
-      </c>
+      <c r="A142" s="3"/>
     </row>
     <row r="143" spans="1:1">
-      <c r="A143" s="3" t="s">
-        <v>120</v>
-      </c>
+      <c r="A143" s="3"/>
     </row>
     <row r="144" spans="1:1">
-      <c r="A144" s="3" t="s">
-        <v>121</v>
-      </c>
+      <c r="A144" s="3"/>
     </row>
     <row r="145" spans="1:1">
-      <c r="A145" s="3" t="s">
-        <v>22</v>
-      </c>
+      <c r="A145" s="3"/>
     </row>
     <row r="146" spans="1:1">
-      <c r="A146" s="3" t="s">
-        <v>122</v>
-      </c>
+      <c r="A146" s="3"/>
     </row>
     <row r="147" spans="1:1">
-      <c r="A147" s="3" t="s">
-        <v>123</v>
-      </c>
+      <c r="A147" s="3"/>
     </row>
     <row r="148" spans="1:1">
-      <c r="A148" s="3" t="s">
-        <v>124</v>
-      </c>
+      <c r="A148" s="3"/>
     </row>
     <row r="149" spans="1:1">
-      <c r="A149" s="3" t="s">
-        <v>125</v>
-      </c>
+      <c r="A149" s="3"/>
     </row>
     <row r="150" spans="1:1">
-      <c r="A150" s="3" t="s">
-        <v>126</v>
-      </c>
+      <c r="A150" s="3"/>
     </row>
     <row r="151" spans="1:1">
-      <c r="A151" s="3" t="s">
-        <v>127</v>
-      </c>
+      <c r="A151" s="3"/>
     </row>
     <row r="152" spans="1:1">
-      <c r="A152" s="3" t="s">
-        <v>128</v>
-      </c>
+      <c r="A152" s="3"/>
     </row>
     <row r="153" spans="1:1">
-      <c r="A153" s="3" t="s">
-        <v>129</v>
-      </c>
+      <c r="A153" s="3"/>
     </row>
     <row r="154" spans="1:1">
-      <c r="A154" s="3" t="s">
-        <v>97</v>
-      </c>
+      <c r="A154" s="3"/>
     </row>
     <row r="155" spans="1:1">
-      <c r="A155" s="3" t="s">
-        <v>130</v>
-      </c>
+      <c r="A155" s="3"/>
     </row>
     <row r="156" spans="1:1">
-      <c r="A156" s="3" t="s">
-        <v>131</v>
-      </c>
+      <c r="A156" s="3"/>
     </row>
     <row r="157" spans="1:1">
-      <c r="A157" s="3" t="s">
-        <v>132</v>
-      </c>
+      <c r="A157" s="3"/>
     </row>
     <row r="158" spans="1:1">
-      <c r="A158" s="3" t="s">
-        <v>133</v>
-      </c>
+      <c r="A158" s="3"/>
     </row>
     <row r="159" spans="1:1">
-      <c r="A159" s="3" t="s">
-        <v>134</v>
-      </c>
+      <c r="A159" s="3"/>
     </row>
     <row r="160" spans="1:1">
-      <c r="A160" s="3" t="s">
-        <v>135</v>
-      </c>
+      <c r="A160" s="3"/>
     </row>
     <row r="161" spans="1:1">
-      <c r="A161" s="3" t="s">
-        <v>136</v>
-      </c>
+      <c r="A161" s="3"/>
     </row>
     <row r="162" spans="1:1">
-      <c r="A162" s="3" t="s">
-        <v>137</v>
-      </c>
+      <c r="A162" s="3"/>
     </row>
     <row r="163" spans="1:1">
-      <c r="A163" s="3" t="s">
-        <v>138</v>
-      </c>
+      <c r="A163" s="3"/>
     </row>
     <row r="164" spans="1:1">
-      <c r="A164" s="3" t="s">
-        <v>80</v>
-      </c>
+      <c r="A164" s="3"/>
     </row>
     <row r="165" spans="1:1">
-      <c r="A165" s="3" t="s">
-        <v>139</v>
-      </c>
+      <c r="A165" s="3"/>
     </row>
     <row r="166" spans="1:1">
-      <c r="A166" s="3" t="s">
-        <v>140</v>
-      </c>
+      <c r="A166" s="3"/>
     </row>
     <row r="167" spans="1:1">
-      <c r="A167" s="3" t="s">
-        <v>141</v>
-      </c>
+      <c r="A167" s="3"/>
     </row>
     <row r="168" spans="1:1">
-      <c r="A168" s="3" t="s">
-        <v>142</v>
-      </c>
+      <c r="A168" s="3"/>
     </row>
     <row r="169" spans="1:1">
-      <c r="A169" s="3" t="s">
-        <v>143</v>
-      </c>
+      <c r="A169" s="3"/>
     </row>
     <row r="170" spans="1:1">
-      <c r="A170" s="3" t="s">
-        <v>144</v>
-      </c>
+      <c r="A170" s="3"/>
     </row>
     <row r="171" spans="1:1">
-      <c r="A171" s="3" t="s">
-        <v>145</v>
-      </c>
+      <c r="A171" s="3"/>
     </row>
     <row r="172" spans="1:1">
-      <c r="A172" s="3" t="s">
-        <v>146</v>
-      </c>
+      <c r="A172" s="3"/>
     </row>
     <row r="173" spans="1:1">
-      <c r="A173" s="3" t="s">
-        <v>147</v>
-      </c>
+      <c r="A173" s="3"/>
     </row>
     <row r="174" spans="1:1">
-      <c r="A174" s="3" t="s">
-        <v>148</v>
-      </c>
+      <c r="A174" s="3"/>
     </row>
     <row r="175" spans="1:1">
-      <c r="A175" s="3" t="s">
-        <v>149</v>
-      </c>
+      <c r="A175" s="3"/>
     </row>
     <row r="176" spans="1:1">
-      <c r="A176" s="3" t="s">
-        <v>150</v>
-      </c>
+      <c r="A176" s="3"/>
     </row>
     <row r="177" spans="1:1">
-      <c r="A177" s="3" t="s">
-        <v>151</v>
-      </c>
+      <c r="A177" s="3"/>
     </row>
     <row r="178" spans="1:1">
-      <c r="A178" s="3" t="s">
-        <v>144</v>
-      </c>
+      <c r="A178" s="3"/>
     </row>
     <row r="179" spans="1:1">
-      <c r="A179" s="3" t="s">
-        <v>152</v>
-      </c>
+      <c r="A179" s="3"/>
     </row>
     <row r="180" spans="1:1">
-      <c r="A180" s="3" t="s">
-        <v>153</v>
-      </c>
+      <c r="A180" s="3"/>
     </row>
     <row r="181" spans="1:1">
-      <c r="A181" s="3" t="s">
-        <v>124</v>
-      </c>
+      <c r="A181" s="3"/>
     </row>
     <row r="182" spans="1:1">
-      <c r="A182" s="3" t="s">
-        <v>154</v>
-      </c>
+      <c r="A182" s="3"/>
     </row>
     <row r="183" spans="1:1">
-      <c r="A183" s="3" t="s">
-        <v>155</v>
-      </c>
+      <c r="A183" s="3"/>
     </row>
     <row r="184" spans="1:1">
-      <c r="A184" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="A184" s="3"/>
     </row>
     <row r="185" spans="1:1">
-      <c r="A185" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="A185" s="3"/>
     </row>
     <row r="186" spans="1:1">
-      <c r="A186" s="3" t="s">
-        <v>156</v>
-      </c>
+      <c r="A186" s="3"/>
     </row>
     <row r="187" spans="1:1">
-      <c r="A187" s="3" t="s">
-        <v>157</v>
-      </c>
+      <c r="A187" s="3"/>
     </row>
     <row r="188" spans="1:1">
-      <c r="A188" s="3" t="s">
-        <v>158</v>
-      </c>
+      <c r="A188" s="3"/>
     </row>
     <row r="189" spans="1:1">
-      <c r="A189" s="3" t="s">
-        <v>159</v>
-      </c>
+      <c r="A189" s="3"/>
     </row>
     <row r="190" spans="1:1">
-      <c r="A190" s="3" t="s">
-        <v>160</v>
-      </c>
+      <c r="A190" s="3"/>
     </row>
     <row r="191" spans="1:1">
-      <c r="A191" s="3" t="s">
-        <v>143</v>
-      </c>
+      <c r="A191" s="3"/>
     </row>
     <row r="192" spans="1:1">
-      <c r="A192" s="3" t="s">
-        <v>161</v>
-      </c>
+      <c r="A192" s="3"/>
     </row>
     <row r="193" spans="1:1">
-      <c r="A193" s="3" t="s">
-        <v>162</v>
-      </c>
+      <c r="A193" s="3"/>
     </row>
     <row r="194" spans="1:1">
-      <c r="A194" s="3" t="s">
-        <v>154</v>
-      </c>
+      <c r="A194" s="3"/>
     </row>
     <row r="195" spans="1:1">
-      <c r="A195" s="3" t="s">
-        <v>163</v>
-      </c>
+      <c r="A195" s="3"/>
     </row>
     <row r="196" spans="1:1">
-      <c r="A196" s="3" t="s">
-        <v>164</v>
-      </c>
+      <c r="A196" s="3"/>
     </row>
     <row r="197" spans="1:1">
-      <c r="A197" s="3" t="s">
-        <v>165</v>
-      </c>
+      <c r="A197" s="3"/>
     </row>
     <row r="198" spans="1:1">
-      <c r="A198" s="3" t="s">
-        <v>166</v>
-      </c>
+      <c r="A198" s="3"/>
     </row>
     <row r="199" spans="1:1">
-      <c r="A199" s="3" t="s">
-        <v>167</v>
-      </c>
+      <c r="A199" s="3"/>
     </row>
     <row r="200" spans="1:1">
-      <c r="A200" s="3" t="s">
-        <v>168</v>
-      </c>
+      <c r="A200" s="3"/>
     </row>
     <row r="201" spans="1:1">
-      <c r="A201" s="3" t="s">
-        <v>76</v>
-      </c>
+      <c r="A201" s="3"/>
     </row>
     <row r="202" spans="1:1">
-      <c r="A202" s="3" t="s">
-        <v>169</v>
-      </c>
+      <c r="A202" s="3"/>
     </row>
     <row r="203" spans="1:1">
-      <c r="A203" s="3" t="s">
-        <v>170</v>
-      </c>
+      <c r="A203" s="3"/>
     </row>
     <row r="204" spans="1:1">
-      <c r="A204" s="3" t="s">
-        <v>75</v>
-      </c>
+      <c r="A204" s="3"/>
     </row>
     <row r="205" spans="1:1">
-      <c r="A205" s="3" t="s">
-        <v>171</v>
-      </c>
+      <c r="A205" s="3"/>
     </row>
     <row r="206" spans="1:1">
-      <c r="A206" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="A206" s="3"/>
     </row>
     <row r="207" spans="1:1">
-      <c r="A207" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="A207" s="3"/>
     </row>
     <row r="208" spans="1:1">
-      <c r="A208" s="3" t="s">
-        <v>173</v>
-      </c>
+      <c r="A208" s="3"/>
     </row>
     <row r="209" spans="1:1">
-      <c r="A209" s="3" t="s">
-        <v>174</v>
-      </c>
+      <c r="A209" s="3"/>
     </row>
     <row r="210" spans="1:1">
-      <c r="A210" s="3" t="s">
-        <v>175</v>
-      </c>
+      <c r="A210" s="3"/>
     </row>
     <row r="211" spans="1:1">
-      <c r="A211" s="3" t="s">
-        <v>176</v>
-      </c>
+      <c r="A211" s="3"/>
     </row>
     <row r="212" spans="1:1">
-      <c r="A212" s="3" t="s">
-        <v>177</v>
-      </c>
+      <c r="A212" s="3"/>
     </row>
     <row r="213" spans="1:1">
-      <c r="A213" s="3" t="s">
-        <v>178</v>
-      </c>
+      <c r="A213" s="3"/>
     </row>
     <row r="214" spans="1:1">
-      <c r="A214" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="A214" s="3"/>
     </row>
     <row r="215" spans="1:1">
-      <c r="A215" s="3" t="s">
-        <v>180</v>
-      </c>
+      <c r="A215" s="3"/>
     </row>
     <row r="216" spans="1:1">
-      <c r="A216" s="3" t="s">
-        <v>181</v>
-      </c>
+      <c r="A216" s="3"/>
     </row>
     <row r="217" spans="1:1">
-      <c r="A217" s="3" t="s">
-        <v>167</v>
-      </c>
+      <c r="A217" s="3"/>
     </row>
     <row r="218" spans="1:1">
-      <c r="A218" s="3" t="s">
-        <v>177</v>
-      </c>
+      <c r="A218" s="3"/>
     </row>
     <row r="219" spans="1:1">
-      <c r="A219" s="3" t="s">
-        <v>182</v>
-      </c>
+      <c r="A219" s="3"/>
     </row>
     <row r="220" spans="1:1">
-      <c r="A220" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="A220" s="3"/>
     </row>
     <row r="221" spans="1:1">
-      <c r="A221" s="3" t="s">
-        <v>183</v>
-      </c>
+      <c r="A221" s="3"/>
     </row>
     <row r="222" spans="1:1">
-      <c r="A222" s="3" t="s">
-        <v>184</v>
-      </c>
+      <c r="A222" s="3"/>
     </row>
     <row r="223" spans="1:1">
-      <c r="A223" s="3" t="s">
-        <v>185</v>
-      </c>
+      <c r="A223" s="3"/>
     </row>
     <row r="224" spans="1:1">
-      <c r="A224" s="3" t="s">
-        <v>181</v>
-      </c>
+      <c r="A224" s="3"/>
     </row>
     <row r="225" spans="1:1">
-      <c r="A225" s="3" t="s">
-        <v>186</v>
-      </c>
+      <c r="A225" s="3"/>
     </row>
     <row r="226" spans="1:1">
-      <c r="A226" s="3" t="s">
-        <v>187</v>
-      </c>
+      <c r="A226" s="3"/>
     </row>
     <row r="227" spans="1:1">
-      <c r="A227" s="3" t="s">
-        <v>188</v>
-      </c>
+      <c r="A227" s="3"/>
     </row>
     <row r="228" spans="1:1">
-      <c r="A228" s="3" t="s">
-        <v>189</v>
-      </c>
+      <c r="A228" s="3"/>
     </row>
     <row r="229" spans="1:1">
-      <c r="A229" s="3" t="s">
-        <v>54</v>
-      </c>
+      <c r="A229" s="3"/>
     </row>
     <row r="230" spans="1:1">
-      <c r="A230" s="3" t="s">
-        <v>177</v>
-      </c>
+      <c r="A230" s="3"/>
     </row>
     <row r="231" spans="1:1">
-      <c r="A231" s="3" t="s">
-        <v>182</v>
-      </c>
+      <c r="A231" s="3"/>
     </row>
     <row r="232" spans="1:1">
-      <c r="A232" s="3" t="s">
-        <v>75</v>
-      </c>
+      <c r="A232" s="3"/>
     </row>
     <row r="233" spans="1:1">
-      <c r="A233" s="3" t="s">
-        <v>190</v>
-      </c>
+      <c r="A233" s="3"/>
     </row>
     <row r="234" spans="1:1">
-      <c r="A234" s="3" t="s">
-        <v>191</v>
-      </c>
+      <c r="A234" s="3"/>
     </row>
     <row r="235" spans="1:1">
-      <c r="A235" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="A235" s="3"/>
     </row>
     <row r="236" spans="1:1">
-      <c r="A236" s="3" t="s">
-        <v>166</v>
-      </c>
+      <c r="A236" s="3"/>
     </row>
     <row r="237" spans="1:1">
-      <c r="A237" s="3" t="s">
-        <v>192</v>
-      </c>
+      <c r="A237" s="3"/>
     </row>
     <row r="238" spans="1:1">
-      <c r="A238" s="3" t="s">
-        <v>181</v>
-      </c>
+      <c r="A238" s="3"/>
     </row>
     <row r="239" spans="1:1">
-      <c r="A239" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="A239" s="3"/>
     </row>
     <row r="240" spans="1:1">
-      <c r="A240" s="3" t="s">
-        <v>193</v>
-      </c>
+      <c r="A240" s="3"/>
     </row>
     <row r="241" spans="1:1">
-      <c r="A241" s="3" t="s">
-        <v>183</v>
-      </c>
+      <c r="A241" s="3"/>
     </row>
     <row r="242" spans="1:1">
-      <c r="A242" s="3" t="s">
-        <v>184</v>
-      </c>
+      <c r="A242" s="3"/>
     </row>
     <row r="243" spans="1:1">
-      <c r="A243" s="3" t="s">
-        <v>178</v>
-      </c>
+      <c r="A243" s="3"/>
     </row>
     <row r="244" spans="1:1">
-      <c r="A244" s="3" t="s">
-        <v>185</v>
-      </c>
+      <c r="A244" s="3"/>
     </row>
     <row r="245" spans="1:1">
-      <c r="A245" s="3" t="s">
-        <v>172</v>
-      </c>
+      <c r="A245" s="3"/>
     </row>
     <row r="246" spans="1:1">
-      <c r="A246" s="3" t="s">
-        <v>194</v>
-      </c>
+      <c r="A246" s="3"/>
     </row>
     <row r="247" spans="1:1">
-      <c r="A247" s="3" t="s">
-        <v>195</v>
-      </c>
+      <c r="A247" s="3"/>
     </row>
     <row r="248" spans="1:1">
-      <c r="A248" s="3" t="s">
-        <v>196</v>
-      </c>
+      <c r="A248" s="3"/>
     </row>
     <row r="249" spans="1:1">
-      <c r="A249" s="3" t="s">
-        <v>197</v>
-      </c>
+      <c r="A249" s="3"/>
     </row>
     <row r="250" spans="1:1">
-      <c r="A250" s="3" t="s">
-        <v>198</v>
-      </c>
+      <c r="A250" s="3"/>
     </row>
     <row r="251" spans="1:1">
-      <c r="A251" s="3" t="s">
-        <v>199</v>
-      </c>
+      <c r="A251" s="3"/>
     </row>
     <row r="252" spans="1:1">
-      <c r="A252" s="3" t="s">
-        <v>200</v>
-      </c>
+      <c r="A252" s="3"/>
     </row>
     <row r="253" spans="1:1">
-      <c r="A253" s="3" t="s">
-        <v>201</v>
-      </c>
+      <c r="A253" s="3"/>
     </row>
     <row r="254" spans="1:1">
-      <c r="A254" s="3" t="s">
-        <v>76</v>
-      </c>
+      <c r="A254" s="3"/>
     </row>
     <row r="255" spans="1:1">
-      <c r="A255" s="3" t="s">
-        <v>202</v>
-      </c>
+      <c r="A255" s="3"/>
     </row>
     <row r="256" spans="1:1">
-      <c r="A256" s="3" t="s">
-        <v>120</v>
-      </c>
+      <c r="A256" s="3"/>
     </row>
     <row r="257" spans="1:1">
-      <c r="A257" s="3" t="s">
-        <v>203</v>
-      </c>
+      <c r="A257" s="3"/>
     </row>
     <row r="258" spans="1:1">
-      <c r="A258" s="3" t="s">
-        <v>168</v>
-      </c>
+      <c r="A258" s="3"/>
     </row>
     <row r="259" spans="1:1">
-      <c r="A259" s="3" t="s">
-        <v>204</v>
-      </c>
+      <c r="A259" s="3"/>
     </row>
     <row r="260" spans="1:1">
-      <c r="A260" s="3" t="s">
-        <v>49</v>
-      </c>
+      <c r="A260" s="3"/>
     </row>
     <row r="261" spans="1:1">
-      <c r="A261" s="3" t="s">
-        <v>169</v>
-      </c>
+      <c r="A261" s="3"/>
     </row>
     <row r="262" spans="1:1">
-      <c r="A262" s="3" t="s">
-        <v>205</v>
-      </c>
+      <c r="A262" s="3"/>
     </row>
     <row r="263" spans="1:1">
-      <c r="A263" s="3" t="s">
-        <v>206</v>
-      </c>
+      <c r="A263" s="3"/>
     </row>
     <row r="264" spans="1:1">
-      <c r="A264" s="3" t="s">
-        <v>207</v>
-      </c>
+      <c r="A264" s="3"/>
     </row>
     <row r="265" spans="1:1">
-      <c r="A265" s="3" t="s">
-        <v>208</v>
-      </c>
+      <c r="A265" s="3"/>
     </row>
     <row r="266" spans="1:1">
-      <c r="A266" s="3" t="s">
-        <v>209</v>
-      </c>
+      <c r="A266" s="3"/>
     </row>
     <row r="267" spans="1:1">
-      <c r="A267" s="3" t="s">
-        <v>210</v>
-      </c>
+      <c r="A267" s="3"/>
     </row>
     <row r="268" spans="1:1">
-      <c r="A268" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="A268" s="3"/>
     </row>
     <row r="269" spans="1:1">
-      <c r="A269" s="3" t="s">
-        <v>211</v>
-      </c>
+      <c r="A269" s="3"/>
     </row>
     <row r="270" spans="1:1">
-      <c r="A270" s="3" t="s">
-        <v>180</v>
-      </c>
+      <c r="A270" s="3"/>
     </row>
     <row r="271" spans="1:1">
-      <c r="A271" s="3" t="s">
-        <v>212</v>
-      </c>
+      <c r="A271" s="3"/>
     </row>
     <row r="272" spans="1:1">
-      <c r="A272" s="3" t="s">
-        <v>176</v>
-      </c>
+      <c r="A272" s="3"/>
     </row>
     <row r="273" spans="1:1">
-      <c r="A273" s="3" t="s">
-        <v>213</v>
-      </c>
+      <c r="A273" s="3"/>
     </row>
     <row r="274" spans="1:1">
-      <c r="A274" s="3" t="s">
-        <v>170</v>
-      </c>
+      <c r="A274" s="3"/>
     </row>
     <row r="275" spans="1:1">
-      <c r="A275" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="A275" s="3"/>
     </row>
     <row r="276" spans="1:1">
-      <c r="A276" s="3" t="s">
-        <v>215</v>
-      </c>
+      <c r="A276" s="3"/>
     </row>
     <row r="277" spans="1:1">
-      <c r="A277" s="3" t="s">
-        <v>216</v>
-      </c>
+      <c r="A277" s="3"/>
     </row>
     <row r="278" spans="1:1">
-      <c r="A278" s="3" t="s">
-        <v>52</v>
-      </c>
+      <c r="A278" s="3"/>
     </row>
     <row r="279" spans="1:1">
-      <c r="A279" s="3" t="s">
-        <v>217</v>
-      </c>
+      <c r="A279" s="3"/>
     </row>
     <row r="280" spans="1:1">
-      <c r="A280" s="3" t="s">
-        <v>218</v>
-      </c>
+      <c r="A280" s="3"/>
     </row>
     <row r="281" spans="1:1">
-      <c r="A281" s="3" t="s">
-        <v>219</v>
-      </c>
+      <c r="A281" s="3"/>
     </row>
     <row r="282" spans="1:1">
-      <c r="A282" s="3" t="s">
-        <v>220</v>
-      </c>
+      <c r="A282" s="3"/>
     </row>
     <row r="283" spans="1:1">
-      <c r="A283" s="3" t="s">
-        <v>221</v>
-      </c>
+      <c r="A283" s="3"/>
     </row>
     <row r="284" spans="1:1">
-      <c r="A284" s="3" t="s">
-        <v>222</v>
-      </c>
+      <c r="A284" s="3"/>
     </row>
     <row r="285" spans="1:1">
-      <c r="A285" s="3" t="s">
-        <v>223</v>
-      </c>
+      <c r="A285" s="3"/>
     </row>
     <row r="286" spans="1:1">
-      <c r="A286" s="3" t="s">
-        <v>224</v>
-      </c>
+      <c r="A286" s="3"/>
     </row>
     <row r="287" spans="1:1">
-      <c r="A287" s="3" t="s">
-        <v>225</v>
-      </c>
+      <c r="A287" s="3"/>
     </row>
     <row r="288" spans="1:1">
-      <c r="A288" s="3" t="s">
-        <v>226</v>
-      </c>
+      <c r="A288" s="3"/>
     </row>
     <row r="289" spans="1:1">
-      <c r="A289" s="3" t="s">
-        <v>227</v>
-      </c>
+      <c r="A289" s="3"/>
     </row>
     <row r="290" spans="1:1">
-      <c r="A290" s="3" t="s">
-        <v>228</v>
-      </c>
+      <c r="A290" s="3"/>
     </row>
     <row r="291" ht="15.2" spans="1:1">
       <c r="A291" s="4"/>

</xml_diff>